<commit_message>
arreglos menores en los codigos
</commit_message>
<xml_diff>
--- a/reporte.xlsx
+++ b/reporte.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,10 +469,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -480,34 +480,34 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>102</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46135.81199074074</v>
+        <v>46135.82646990741</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G2" t="n">
-        <v>120000</v>
+        <v>400000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Camiseta Adidas</t>
+          <t>Chaquetas de Cuero</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Andrea</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -515,55 +515,55 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>46135.8115625</v>
+        <v>46135.82606481481</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G3" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Medias tobilleras</t>
+          <t>Sandalias</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Andrea</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>entrada</t>
+          <t>salida</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>102</v>
+        <v>21</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>46135.81043981481</v>
+        <v>46135.81199074074</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>400000</v>
+        <v>120000</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Chaquetas de Cuero</t>
+          <t>Camiseta Adidas</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -574,31 +574,31 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>102</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>46132.60282407407</v>
+        <v>46135.8115625</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>135000</v>
+        <v>10000</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>camisetas nike</t>
+          <t>Medias tobilleras</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -609,10 +609,10 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -620,20 +620,20 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>102</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>46132.59940972222</v>
+        <v>46135.81043981481</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>120000</v>
+        <v>400000</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>puma</t>
+          <t>Chaquetas de Cuero</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -644,10 +644,10 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -655,20 +655,20 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>46132.59643518519</v>
+        <v>46132.60282407407</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>90000</v>
+        <v>135000</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>camisetas nike</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -679,21 +679,21 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" t="n">
         <v>2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>46132.53179398148</v>
+        <v>46132.59940972222</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
@@ -714,45 +714,45 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>entrada</t>
+          <t>salida</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>46132.51681712963</v>
+        <v>46132.59643518519</v>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>90000</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Camiseta Adidas</t>
+          <t>pantalon levi's</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>andres</t>
+          <t>Admin</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -760,20 +760,20 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>46129.4031712963</v>
+        <v>46132.53179398148</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>puma</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -784,10 +784,10 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -795,31 +795,31 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>46129.40282407407</v>
+        <v>46132.51681712963</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>Camiseta Adidas</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>andres</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B12" t="n">
         <v>3</v>
@@ -830,10 +830,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>46126.70535879629</v>
+        <v>46129.4031712963</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -854,21 +854,21 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B13" t="n">
         <v>3</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>12</v>
+        <v>120</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>46126.6990162037</v>
+        <v>46129.40282407407</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
@@ -889,21 +889,21 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B14" t="n">
         <v>3</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>entrada</t>
+          <t>salida</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>46126.6985300926</v>
+        <v>46126.70535879629</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
@@ -924,21 +924,21 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B15" t="n">
         <v>3</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>entrada</t>
+          <t>salida</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>46126.69717592592</v>
+        <v>46126.6990162037</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
@@ -959,21 +959,21 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B16" t="n">
         <v>3</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>46126.69645833333</v>
+        <v>46126.6985300926</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
@@ -994,21 +994,21 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B17" t="n">
         <v>3</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>46126.69400462963</v>
+        <v>46126.69717592592</v>
       </c>
       <c r="F17" t="n">
         <v>1</v>
@@ -1029,10 +1029,10 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1040,10 +1040,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>46126.64710648148</v>
+        <v>46126.69645833333</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>puma</t>
+          <t>pantalon levi's</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1064,21 +1064,21 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>entrada</t>
+          <t>salida</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>101</v>
+        <v>10</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>46126.64673611111</v>
+        <v>46126.69400462963</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
@@ -1088,10 +1088,80 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>51</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>46126.64710648148</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>puma</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>entrada</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>101</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>46126.64673611111</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>puma</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>

</xml_diff>

<commit_message>
Ultimos arreglos del sistema
</commit_message>
<xml_diff>
--- a/reporte.xlsx
+++ b/reporte.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,10 +469,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -480,34 +480,34 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46135.82646990741</v>
+        <v>46149.46357638889</v>
       </c>
       <c r="F2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>400000</v>
+        <v>10000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Chaquetas de Cuero</t>
+          <t>Medias tobilleras</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Andrea</t>
+          <t>Admin</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -518,48 +518,48 @@
         <v>50</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>46135.82606481481</v>
+        <v>46149.46299768519</v>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>30000</v>
+        <v>20000</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Sandalias</t>
+          <t>camisas</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Andrea</t>
+          <t>Admin</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="B4" t="n">
         <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>46135.81199074074</v>
+        <v>46146.82917824074</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>120000</v>
+        <v>50000</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -568,16 +568,16 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>andres</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -585,20 +585,20 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>46135.8115625</v>
+        <v>46146.75503472222</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Medias tobilleras</t>
+          <t>botas para la lluvia</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -609,10 +609,10 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -620,20 +620,20 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>46135.81043981481</v>
+        <v>46146.73230324074</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>400000</v>
+        <v>30000</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Chaquetas de Cuero</t>
+          <t>Ropa interior mujer</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -644,66 +644,66 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>46146.72921296296</v>
+      </c>
+      <c r="F7" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="1" t="n">
-        <v>46132.60282407407</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
       <c r="G7" t="n">
-        <v>135000</v>
+        <v>345000</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>camisetas nike</t>
+          <t>buzos de f1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>andres</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>entrada</t>
+          <t>salida</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>46132.59940972222</v>
+        <v>46146.72841435186</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>120000</v>
+        <v>400000</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>puma</t>
+          <t>Chaquetas de Cuero</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -714,31 +714,31 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>46132.59643518519</v>
+        <v>46146.72774305556</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>90000</v>
+        <v>30000</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>Ropa interior de hombre</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -749,10 +749,10 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -760,10 +760,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>46132.53179398148</v>
+        <v>46146.72728009259</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -773,7 +773,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>puma</t>
+          <t>Camiseta Adidas</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -784,10 +784,10 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -795,45 +795,45 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>46132.51681712963</v>
+        <v>46146.72643518518</v>
       </c>
       <c r="F11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Camiseta Adidas</t>
+          <t>Ropa interior de hombre</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>andres</t>
+          <t>Admin</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>46129.4031712963</v>
+        <v>46146.72546296296</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -843,7 +843,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>Ropa interior de hombre</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -854,10 +854,10 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -865,20 +865,20 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>46129.40282407407</v>
+        <v>46143.41196759259</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>Sandalias</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -889,10 +889,10 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -900,34 +900,34 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>46126.70535879629</v>
+        <v>46141.77214120371</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>Sandalias</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>andres</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -935,20 +935,20 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>46126.6990162037</v>
+        <v>46141.77116898148</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>Medias tobilleras</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -959,10 +959,10 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -970,20 +970,20 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>46126.6985300926</v>
+        <v>46141.77081018518</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>345000</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>buzos de f1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -994,80 +994,80 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
+        <v>20</v>
+      </c>
+      <c r="B17" t="n">
         <v>5</v>
       </c>
-      <c r="B17" t="n">
-        <v>3</v>
-      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>entrada</t>
+          <t>salida</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>15</v>
+        <v>102</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>46126.69717592592</v>
+        <v>46135.82646990741</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>400000</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>Chaquetas de Cuero</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Andrea</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>46126.69645833333</v>
+        <v>46135.82606481481</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>Sandalias</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Andrea</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1075,20 +1075,20 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>46126.69400462963</v>
+        <v>46135.81199074074</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>pantalon levi's</t>
+          <t>Camiseta Adidas</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1099,31 +1099,31 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>salida</t>
+          <t>entrada</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>51</v>
+        <v>102</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>46126.64710648148</v>
+        <v>46135.8115625</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>puma</t>
+          <t>Medias tobilleras</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1134,34 +1134,559 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>entrada</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>102</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>46135.81043981481</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>400000</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Chaquetas de Cuero</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>46132.60282407407</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>135000</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>camisetas nike</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>14</v>
+      </c>
+      <c r="B23" t="n">
         <v>2</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>entrada</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>entrada</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>46132.59940972222</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>120000</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>puma</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>46132.59643518519</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>90000</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>46132.53179398148</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>120000</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>puma</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>entrada</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>20</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>46132.51681712963</v>
+      </c>
+      <c r="F26" t="n">
+        <v>5</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Camiseta Adidas</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>andres</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>50</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>46129.4031712963</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>entrada</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>120</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>46129.40282407407</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>8</v>
+      </c>
+      <c r="B29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>15</v>
+      </c>
+      <c r="E29" s="1" t="n">
+        <v>46126.70535879629</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>7</v>
+      </c>
+      <c r="B30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>12</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>46126.6990162037</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>6</v>
+      </c>
+      <c r="B31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>entrada</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>12</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>46126.6985300926</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>entrada</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>15</v>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>46126.69717592592</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>46126.69645833333</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>3</v>
+      </c>
+      <c r="B34" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>46126.69400462963</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>pantalon levi's</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>51</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>46126.64710648148</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>puma</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>entrada</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
         <v>101</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E36" s="1" t="n">
         <v>46126.64673611111</v>
       </c>
-      <c r="F21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" t="n">
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="n">
         <v>0</v>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>puma</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>

</xml_diff>